<commit_message>
delete default secretkey add default db sevẻ
</commit_message>
<xml_diff>
--- a/CHECKLIST_TEST.xlsx
+++ b/CHECKLIST_TEST.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="14100"/>
+    <workbookView windowHeight="15360"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist Test" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="187">
   <si>
     <t>Mã test</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Health</t>
   </si>
   <si>
-    <t>Kiểm tra server còn sống</t>
+    <t>Kiểm tra server hoạt động</t>
   </si>
   <si>
     <t>GET /health</t>
@@ -74,6 +74,9 @@
     <t>200 {"status": "ok"}</t>
   </si>
   <si>
+    <t>Pass</t>
+  </si>
+  <si>
     <t>TC-002</t>
   </si>
   <si>
@@ -104,6 +107,12 @@
     <t>409 Conflict</t>
   </si>
   <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Vì khi kiểm tra database phát hiện user.email == email -&gt; 409</t>
+  </si>
+  <si>
     <t>TC-004</t>
   </si>
   <si>
@@ -116,6 +125,9 @@
     <t>422 Unprocessable</t>
   </si>
   <si>
+    <t xml:space="preserve">Khi Field kiểm tra dữ liệu Min là 6 -&gt; 422 </t>
+  </si>
+  <si>
     <t>TC-005</t>
   </si>
   <si>
@@ -123,6 +135,9 @@
   </si>
   <si>
     <t>{"email": "x@test.com"} (thiếu full_name, password)</t>
+  </si>
+  <si>
+    <t>Kiểm tra bằng Field thì đều kiểm tra độ dài của full_name &gt; 2 và password &gt; 6</t>
   </si>
   <si>
     <t>TC-006</t>
@@ -588,7 +603,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -600,13 +615,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1080,148 +1088,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1591,8 +1599,8 @@
     <col min="4" max="4" width="41.6640625" customWidth="1"/>
     <col min="5" max="5" width="45.1796875" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="7" max="7" width="14.578125" customWidth="1"/>
+    <col min="8" max="8" width="68.8125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" spans="1:8">
@@ -1640,730 +1648,754 @@
       <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="3" ht="34" spans="1:8">
       <c r="A3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
         <v>14</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" ht="17" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="5" ht="17" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>27</v>
+      <c r="H5" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>27</v>
+      <c r="G6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" ht="17" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" ht="17" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" ht="17" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" ht="17" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" ht="17" spans="1:8">
       <c r="A12" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" ht="17" spans="1:8">
       <c r="A13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" ht="17" spans="1:8">
       <c r="A14" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" ht="17" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" ht="17" spans="1:8">
       <c r="A16" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" ht="17" spans="1:6">
       <c r="A17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="C17" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" ht="17" spans="1:6">
       <c r="A18" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" ht="17" spans="1:6">
       <c r="A19" s="2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" ht="17" spans="1:6">
       <c r="A20" s="2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" ht="17" spans="1:6">
       <c r="A21" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" ht="17" spans="1:6">
       <c r="A22" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="C22" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" ht="17" spans="1:6">
       <c r="A23" s="2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" ht="17" spans="1:6">
       <c r="A24" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" ht="17" spans="1:6">
       <c r="A25" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="C25" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26" ht="17" spans="1:6">
       <c r="A26" s="2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27" ht="34" spans="1:6">
       <c r="A27" s="2" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" ht="17" spans="1:6">
       <c r="A28" s="2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="29" ht="34" spans="1:6">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="29" ht="17" spans="1:6">
       <c r="A29" s="2" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="30" ht="34" spans="1:6">
       <c r="A30" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" ht="17" spans="1:6">
       <c r="A31" s="2" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="32" ht="17" spans="1:6">
       <c r="A32" s="2" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33" ht="17" spans="1:6">
       <c r="A33" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="C33" s="2" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="34" ht="17" spans="1:6">
       <c r="A34" s="2" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="35" ht="17" spans="1:6">
       <c r="A35" s="2" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="36" ht="17" spans="1:6">
       <c r="A36" s="2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" ht="34" spans="1:6">
       <c r="A37" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>168</v>
-      </c>
       <c r="C37" s="2" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="38" ht="17" spans="1:6">
       <c r="A38" s="2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="3" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -2377,7 +2409,7 @@
     <mergeCell ref="A40:D40"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="G2:G38">
+    <dataValidation type="list" allowBlank="1" sqref="G3 G4:G38">
       <formula1>"Pass,Fail,Chưa test"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>